<commit_message>
Encode NOTE-37: combine same-item receipts; mark 125315 Success.
Kyle finished 10107 live (24126 8@$33 + 24127 13@$33 = 21@$33=$693).
GET-only — do not re-Select Receipts. HOLDs 10108/10111 left alone.
Sheet Why notes Kyle's 2026-09-17 finish. No Mail.Send. invent=false.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-16-jpsteel.xlsx
+++ b/runs/AP-run-2026-09-16-jpsteel.xlsx
@@ -46,12 +46,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -569,12 +569,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>Success</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>HOLD (receipt): Select Receipts blocked-400 on same-PO-line split 24126 8@$33 + 24127 13@$33 (PDF 21@$33=$693, verification=693.00). Header+PDF on batch 716. Do not invent Success. @Shawn McKibben can Select Receipts in GI. Outlook Entered with issues. Flag status=entered-with-issues.</t>
+          <t>Kyle finished Select Receipts 2026-09-17 (NOTE-37: combine same-item same-unit-cost 24126 8@33.0; 24127 13@33.0 = PDF 21@$33=$693). Live GET 10107 Invoice_Amount=693.0 verification=693.0 Type 3 vendor 100 batch 716. Did not Select Receipts / edit / re-finish — Kyle's live state left alone. Outlook left as Kyle set (not re-stamped).</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -607,7 +607,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
@@ -636,7 +636,7 @@
       <c r="E3" s="2" t="n">
         <v>1580.73</v>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
@@ -705,7 +705,7 @@
       <c r="E4" s="2" t="n">
         <v>2530</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Success</t>
         </is>
@@ -774,7 +774,7 @@
       <c r="E5" s="2" t="n">
         <v>832.03</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Success</t>
         </is>
@@ -843,7 +843,7 @@
       <c r="E6" s="2" t="n">
         <v>1130.4</v>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>

</xml_diff>

<commit_message>
Finish JPSteel 10108 and 10111 with in-gate rounding PPV.
Live GET: 10108 Invoice_Amount 1580.73 after PPV -$0.10;
10111 Invoice_Amount 1130.40 after PPV +$0.06. Outlook Entered in AI.
10107 left read-only. Sheet 5 Success / 0 HOLD. No Mail.Send.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/AP-run-2026-09-16-jpsteel.xlsx
+++ b/runs/AP-run-2026-09-16-jpsteel.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,11 +49,6 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,7 +62,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -76,9 +71,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -636,14 +628,14 @@
       <c r="E3" s="2" t="n">
         <v>1580.73</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>HOLD after live GET of 10108: PDF/verification=$1,580.73 posted=$1,580.83 ($0.10 unit-rounding). Receipts 24128 1445in @0.7709 + 24129 1245in @0.375 on PO 59154 (partial of 14400/14940; cut length 289"/249" was not qty). Do not invent Success. Outlook Entered with issues.</t>
+          <t>NOTE-38: signed PPV -$0.10 posted so Invoice_Amount hits PDF $1,580.73 (was $1,580.83). Receipts 24128 1445@0.7709; 24129 1245@0.375 already matched. Live GET 10108 Invoice_Amount=1580.73 verification=1580.73 Type 3. Outlook Entered in AI. Success.</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -661,7 +653,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>-0.10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -676,7 +668,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
@@ -712,7 +704,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=59104. Select Receipts 24122 2@115.0; 24123 20@115.0 on PO 59104. Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[24122, 24123] fees=none ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59104. Select Receipts 24122 2@115.0; 24123 20@115.0 on PO 59104. Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -781,7 +773,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Finished bill (Invoice_Type 3). Header PO set=59018. Select Receipts 23706 520@0.2708; 23707 2880@0.24 on PO 59018. Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Finish Select Receipts selected ids=[23706, 23707] fees=none ppv=none. Flag status=entered-in-ai.</t>
+          <t>Finished bill (Invoice_Type 3). Header PO set=59018. Select Receipts 23706 520@0.2708; 23707 2880@0.24 on PO 59018. Fees=none (Additional Charge Fees id 11, not PPV). PPV=none. Attach status=attached. Flag status=entered-in-ai.</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -843,14 +835,14 @@
       <c r="E6" s="2" t="n">
         <v>1130.4</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HOLD after live GET of 10111: PDF/verification=$1,130.40 posted=$1,130.34 ($0.06). Receipts 23559 576in @0.6598 + 23560 864in @0.8684 on PO 58937 lines 03/04 (line-order swap vs SO 1/2). Do not invent Success. Outlook Entered with issues.</t>
+          <t>NOTE-38: signed PPV +$0.06 posted so Invoice_Amount hits PDF $1,130.40 (was $1,130.34). Receipts 23559 576@0.6598; 23560 864@0.8684 already matched. Live GET 10111 Invoice_Amount=1130.40 verification=1130.40 Type 3. Outlook Entered in AI. Success.</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -868,7 +860,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -883,7 +875,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>entered-with-issues</t>
+          <t>entered-in-ai</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr"/>

</xml_diff>